<commit_message>
Add open-position recommendations to Next Step sheet
</commit_message>
<xml_diff>
--- a/adaptive_ev_calculator.xlsx
+++ b/adaptive_ev_calculator.xlsx
@@ -19,7 +19,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.00000"/>
+  </numFmts>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
@@ -72,7 +74,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -82,6 +84,7 @@
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -8169,7 +8172,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -8245,6 +8248,26 @@
           <t>Причина</t>
         </is>
       </c>
+      <c r="K1" s="6" t="inlineStr">
+        <is>
+          <t>Открыть позицию?</t>
+        </is>
+      </c>
+      <c r="L1" s="6" t="inlineStr">
+        <is>
+          <t>Направление открытия</t>
+        </is>
+      </c>
+      <c r="M1" s="6" t="inlineStr">
+        <is>
+          <t>Лот открытия</t>
+        </is>
+      </c>
+      <c r="N1" s="6" t="inlineStr">
+        <is>
+          <t>Цена открытия</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -8290,6 +8313,22 @@
         <f>IF(I2="ДА","Риск превышен: survival/маржа/просадка","Нормальный цикл")</f>
         <v/>
       </c>
+      <c r="K2">
+        <f>IF(AND(Расчеты!B11="ДА",I2="НЕТ"),"ДА","НЕТ")</f>
+        <v/>
+      </c>
+      <c r="L2">
+        <f>IF(K2="НЕТ","-",IF(D2="BUY (Рекомендации для выбранной BUY)","BUY","SELL"))</f>
+        <v/>
+      </c>
+      <c r="M2" s="5">
+        <f>IF(K2="НЕТ",0,ROUND(MAX(0.01,F2),2))</f>
+        <v/>
+      </c>
+      <c r="N2" s="7">
+        <f>IF(K2="НЕТ",0,IF(L2="BUY",Ввод!B14,Ввод!B13))</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -8335,6 +8374,22 @@
         <f>IF(I3="ДА","Риск превышен: survival/маржа/просадка","Нормальный цикл")</f>
         <v/>
       </c>
+      <c r="K3">
+        <f>IF(AND(Расчеты!B11="ДА",I3="НЕТ"),"ДА","НЕТ")</f>
+        <v/>
+      </c>
+      <c r="L3">
+        <f>IF(K3="НЕТ","-",IF(D3="BUY (Рекомендации для выбранной BUY)","BUY","SELL"))</f>
+        <v/>
+      </c>
+      <c r="M3" s="5">
+        <f>IF(K3="НЕТ",0,ROUND(MAX(0.01,F3),2))</f>
+        <v/>
+      </c>
+      <c r="N3" s="7">
+        <f>IF(K3="НЕТ",0,IF(L3="BUY",Ввод!B14,Ввод!B13))</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -8380,6 +8435,22 @@
         <f>IF(I4="ДА","Риск превышен: survival/маржа/просадка","Нормальный цикл")</f>
         <v/>
       </c>
+      <c r="K4">
+        <f>IF(AND(Расчеты!B11="ДА",I4="НЕТ"),"ДА","НЕТ")</f>
+        <v/>
+      </c>
+      <c r="L4">
+        <f>IF(K4="НЕТ","-",IF(D4="BUY (Рекомендации для выбранной BUY)","BUY","SELL"))</f>
+        <v/>
+      </c>
+      <c r="M4" s="5">
+        <f>IF(K4="НЕТ",0,ROUND(MAX(0.01,F4),2))</f>
+        <v/>
+      </c>
+      <c r="N4" s="7">
+        <f>IF(K4="НЕТ",0,IF(L4="BUY",Ввод!B14,Ввод!B13))</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -8423,6 +8494,22 @@
       </c>
       <c r="J5">
         <f>IF(I5="ДА","Риск превышен: survival/маржа/просадка","Нормальный цикл")</f>
+        <v/>
+      </c>
+      <c r="K5">
+        <f>IF(AND(Расчеты!B11="ДА",I5="НЕТ"),"ДА","НЕТ")</f>
+        <v/>
+      </c>
+      <c r="L5">
+        <f>IF(K5="НЕТ","-",IF(D5="BUY (Рекомендации для выбранной BUY)","BUY","SELL"))</f>
+        <v/>
+      </c>
+      <c r="M5" s="5">
+        <f>IF(K5="НЕТ",0,ROUND(MAX(0.01,F5),2))</f>
+        <v/>
+      </c>
+      <c r="N5" s="7">
+        <f>IF(K5="НЕТ",0,IF(L5="BUY",Ввод!B14,Ввод!B13))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix open-position recommendation logic in Next Step sheet
</commit_message>
<xml_diff>
--- a/adaptive_ev_calculator.xlsx
+++ b/adaptive_ev_calculator.xlsx
@@ -8314,7 +8314,7 @@
         <v/>
       </c>
       <c r="K2">
-        <f>IF(AND(Расчеты!B11="ДА",I2="НЕТ"),"ДА","НЕТ")</f>
+        <f>IF(AND(F2&gt;0,I2="НЕТ"),"ДА","НЕТ")</f>
         <v/>
       </c>
       <c r="L2">
@@ -8326,7 +8326,7 @@
         <v/>
       </c>
       <c r="N2" s="7">
-        <f>IF(K2="НЕТ",0,IF(L2="BUY",Ввод!B14,Ввод!B13))</f>
+        <f>IF(K2="НЕТ",0,B2)</f>
         <v/>
       </c>
     </row>
@@ -8375,7 +8375,7 @@
         <v/>
       </c>
       <c r="K3">
-        <f>IF(AND(Расчеты!B11="ДА",I3="НЕТ"),"ДА","НЕТ")</f>
+        <f>IF(AND(F3&gt;0,I3="НЕТ"),"ДА","НЕТ")</f>
         <v/>
       </c>
       <c r="L3">
@@ -8387,7 +8387,7 @@
         <v/>
       </c>
       <c r="N3" s="7">
-        <f>IF(K3="НЕТ",0,IF(L3="BUY",Ввод!B14,Ввод!B13))</f>
+        <f>IF(K3="НЕТ",0,B3)</f>
         <v/>
       </c>
     </row>
@@ -8436,7 +8436,7 @@
         <v/>
       </c>
       <c r="K4">
-        <f>IF(AND(Расчеты!B11="ДА",I4="НЕТ"),"ДА","НЕТ")</f>
+        <f>IF(AND(F4&gt;0,I4="НЕТ"),"ДА","НЕТ")</f>
         <v/>
       </c>
       <c r="L4">
@@ -8448,7 +8448,7 @@
         <v/>
       </c>
       <c r="N4" s="7">
-        <f>IF(K4="НЕТ",0,IF(L4="BUY",Ввод!B14,Ввод!B13))</f>
+        <f>IF(K4="НЕТ",0,B4)</f>
         <v/>
       </c>
     </row>
@@ -8497,7 +8497,7 @@
         <v/>
       </c>
       <c r="K5">
-        <f>IF(AND(Расчеты!B11="ДА",I5="НЕТ"),"ДА","НЕТ")</f>
+        <f>IF(AND(F5&gt;0,I5="НЕТ"),"ДА","НЕТ")</f>
         <v/>
       </c>
       <c r="L5">
@@ -8509,7 +8509,7 @@
         <v/>
       </c>
       <c r="N5" s="7">
-        <f>IF(K5="НЕТ",0,IF(L5="BUY",Ввод!B14,Ввод!B13))</f>
+        <f>IF(K5="НЕТ",0,B5)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Add new-position lot/price recommendations to EV calculator
</commit_message>
<xml_diff>
--- a/adaptive_ev_calculator.xlsx
+++ b/adaptive_ev_calculator.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Позиции" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Расчеты" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Следующий шаг" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Новые позиции" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -74,7 +75,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -85,6 +86,7 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -8516,4 +8518,165 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="28" customWidth="1" min="12" max="12"/>
+    <col width="28" customWidth="1" min="13" max="13"/>
+    <col width="28" customWidth="1" min="14" max="14"/>
+    <col width="28" customWidth="1" min="15" max="15"/>
+    <col width="28" customWidth="1" min="16" max="16"/>
+    <col width="28" customWidth="1" min="17" max="17"/>
+    <col width="28" customWidth="1" min="18" max="18"/>
+    <col width="28" customWidth="1" min="19" max="19"/>
+    <col width="28" customWidth="1" min="20" max="20"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Сценарий</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Триггер</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Рекомендация открытия</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>Направление</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>Рекомендуемый лот</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>Рекомендуемая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>Оценка маржи, USD</t>
+        </is>
+      </c>
+      <c r="H1" s="6" t="inlineStr">
+        <is>
+          <t>Свободная маржа после открытия, USD</t>
+        </is>
+      </c>
+      <c r="I1" s="6" t="inlineStr">
+        <is>
+          <t>Комментарий</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Пробой вверх (+Δ)</t>
+        </is>
+      </c>
+      <c r="B2">
+        <f>IF(Ввод!B12&gt;=Расчеты!B5+Ввод!B18,"ДА","НЕТ")</f>
+        <v/>
+      </c>
+      <c r="C2">
+        <f>IF(B2="ДА","ОТКРЫТЬ","ЖДАТЬ")</f>
+        <v/>
+      </c>
+      <c r="D2">
+        <f>IF(A2="Пробой вверх (+Δ)","BUY","SELL")</f>
+        <v/>
+      </c>
+      <c r="E2" s="5">
+        <f>IF(C2&lt;&gt;"ОТКРЫТЬ",0,ROUND(MAX(0.01,MIN(Ввод!B20*0.01*Ввод!B23,(Ввод!B10*Ввод!B22/100-Расчеты!B13)*Ввод!B7/(Ввод!B6*Ввод!B12))),2))</f>
+        <v/>
+      </c>
+      <c r="F2" s="7">
+        <f>IF(E2=0,0,IF(D2="BUY",Ввод!B14,Ввод!B13))</f>
+        <v/>
+      </c>
+      <c r="G2" s="8">
+        <f>IF(E2=0,0,E2*Ввод!B6*F2/Ввод!B7)</f>
+        <v/>
+      </c>
+      <c r="H2" s="8">
+        <f>Ввод!B10-G2</f>
+        <v/>
+      </c>
+      <c r="I2">
+        <f>IF(E2=0,"Нет сигнала или лимит маржи","Открыть только при рыночном подтверждении")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Пробой вниз (-Δ)</t>
+        </is>
+      </c>
+      <c r="B3">
+        <f>IF(Ввод!B12&lt;=Расчеты!B5-Ввод!B18,"ДА","НЕТ")</f>
+        <v/>
+      </c>
+      <c r="C3">
+        <f>IF(B3="ДА","ОТКРЫТЬ","ЖДАТЬ")</f>
+        <v/>
+      </c>
+      <c r="D3">
+        <f>IF(A3="Пробой вверх (+Δ)","BUY","SELL")</f>
+        <v/>
+      </c>
+      <c r="E3" s="5">
+        <f>IF(C3&lt;&gt;"ОТКРЫТЬ",0,ROUND(MAX(0.01,MIN(Ввод!B20*0.01*Ввод!B23,(Ввод!B10*Ввод!B22/100-Расчеты!B13)*Ввод!B7/(Ввод!B6*Ввод!B12))),2))</f>
+        <v/>
+      </c>
+      <c r="F3" s="7">
+        <f>IF(E3=0,0,IF(D3="BUY",Ввод!B14,Ввод!B13))</f>
+        <v/>
+      </c>
+      <c r="G3" s="8">
+        <f>IF(E3=0,0,E3*Ввод!B6*F3/Ввод!B7)</f>
+        <v/>
+      </c>
+      <c r="H3" s="8">
+        <f>Ввод!B10-G3</f>
+        <v/>
+      </c>
+      <c r="I3">
+        <f>IF(E3=0,"Нет сигнала или лимит маржи","Открыть только при рыночном подтверждении")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Align EV system with FSM risk-controller manual and adaptive k
</commit_message>
<xml_diff>
--- a/adaptive_ev_calculator.xlsx
+++ b/adaptive_ev_calculator.xlsx
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -702,6 +702,16 @@
         <v>1</v>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>k_min</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
@@ -722,6 +732,27 @@
       <c r="B26">
         <f>IF(OR(Расчеты!B9="FAIL",Расчеты!B14&gt;B22,Расчеты!B16&lt;-B21),"СТРЕСС/СОКРАЩЕНИЕ","НОРМА")</f>
         <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Состояние FSM</t>
+        </is>
+      </c>
+      <c r="B27">
+        <f>Расчеты!B22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Смещение bias, %</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -7918,7 +7949,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -8160,6 +8191,61 @@
       </c>
       <c r="B20">
         <f>IFERROR(INDEX(Позиции!D$2:D$201,MATCH(B18,Позиции!A$2:A$201,0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Экспозиция E=|Lb-Ls|</t>
+        </is>
+      </c>
+      <c r="B21">
+        <f>ABS(B1-B2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Норм. волатильность v=ATR/Δ</t>
+        </is>
+      </c>
+      <c r="B22">
+        <f>IF(Ввод!B18=0,0,Ввод!B16/Ввод!B18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>k(ATR)</t>
+        </is>
+      </c>
+      <c r="B23">
+        <f>Ввод!B24+(Ввод!B25-Ввод!B24)*EXP(-Ввод!B26*B24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>k адаптивный</t>
+        </is>
+      </c>
+      <c r="B24">
+        <f>MAX(Ввод!B24,MIN(Ввод!B25,B23*(1-0.5*B22/MAX(Ввод!B27,0.0001))*(1-0.5*MAX(0,-B16)/MAX(Ввод!B21,0.0001))*(1-0.4*B2/MAX(1,1))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Режим FSM</t>
+        </is>
+      </c>
+      <c r="B25">
+        <f>IF(OR(B14&gt;Ввод!B22,B16&lt;-Ввод!B21),"ESCAPE",IF(OR(B23&gt;0.7*Ввод!B27,B14&gt;0.7*Ввод!B22),"STRESS","FLOW"))</f>
         <v/>
       </c>
     </row>
@@ -8621,7 +8707,7 @@
         <v/>
       </c>
       <c r="F2" s="7">
-        <f>IF(E2=0,0,IF(D2="BUY",Ввод!B14,Ввод!B13))</f>
+        <f>IF(E2=0,0,IF(D2="BUY",Ввод!B14-Ввод!B18*(Ввод!B28/100),Ввод!B13+Ввод!B18*(Ввод!B28/100)))</f>
         <v/>
       </c>
       <c r="G2" s="8">
@@ -8660,7 +8746,7 @@
         <v/>
       </c>
       <c r="F3" s="7">
-        <f>IF(E3=0,0,IF(D3="BUY",Ввод!B14,Ввод!B13))</f>
+        <f>IF(E3=0,0,IF(D3="BUY",Ввод!B14-Ввод!B18*(Ввод!B28/100),Ввод!B13+Ввод!B18*(Ввод!B28/100)))</f>
         <v/>
       </c>
       <c r="G3" s="8">

</xml_diff>

<commit_message>
Refactor 'Следующий шаг' and 'Новые позиции' formulas to remove duplicates and align FSM logic
</commit_message>
<xml_diff>
--- a/adaptive_ev_calculator.xlsx
+++ b/adaptive_ev_calculator.xlsx
@@ -8260,7 +8260,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -8298,62 +8298,62 @@
       </c>
       <c r="C1" s="6" t="inlineStr">
         <is>
-          <t>ID Позиции</t>
+          <t>Текущее состояние FSM</t>
         </is>
       </c>
       <c r="D1" s="6" t="inlineStr">
         <is>
-          <t>Для BUY/SELL</t>
+          <t>Что делать с локом</t>
         </is>
       </c>
       <c r="E1" s="6" t="inlineStr">
         <is>
-          <t>Направление шага</t>
+          <t>Реком. коэффициент k</t>
         </is>
       </c>
       <c r="F1" s="6" t="inlineStr">
         <is>
-          <t>Рекоменд. лот</t>
+          <t>Реком. лот действия</t>
         </is>
       </c>
       <c r="G1" s="6" t="inlineStr">
         <is>
-          <t>Действие</t>
+          <t>Частичное закрытие BUY</t>
         </is>
       </c>
       <c r="H1" s="6" t="inlineStr">
         <is>
-          <t>Частично закрыть лот</t>
+          <t>Частичное закрытие SELL</t>
         </is>
       </c>
       <c r="I1" s="6" t="inlineStr">
         <is>
-          <t>Полностью закрыть?</t>
+          <t>Открыть новый цикл?</t>
         </is>
       </c>
       <c r="J1" s="6" t="inlineStr">
         <is>
+          <t>Направление нового цикла</t>
+        </is>
+      </c>
+      <c r="K1" s="6" t="inlineStr">
+        <is>
+          <t>Лот нового цикла</t>
+        </is>
+      </c>
+      <c r="L1" s="6" t="inlineStr">
+        <is>
+          <t>Цена нового цикла</t>
+        </is>
+      </c>
+      <c r="M1" s="6" t="inlineStr">
+        <is>
           <t>Причина</t>
         </is>
       </c>
-      <c r="K1" s="6" t="inlineStr">
-        <is>
-          <t>Открыть позицию?</t>
-        </is>
-      </c>
-      <c r="L1" s="6" t="inlineStr">
-        <is>
-          <t>Направление открытия</t>
-        </is>
-      </c>
-      <c r="M1" s="6" t="inlineStr">
-        <is>
-          <t>Лот открытия</t>
-        </is>
-      </c>
       <c r="N1" s="6" t="inlineStr">
         <is>
-          <t>Цена открытия</t>
+          <t>Стоп-условие</t>
         </is>
       </c>
     </row>
@@ -8368,236 +8368,110 @@
         <v/>
       </c>
       <c r="C2">
-        <f>IF(D2="BUY (Рекомендации для выбранной BUY)",Расчеты!B17,Расчеты!B18)</f>
-        <v/>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>BUY (Рекомендации для выбранной BUY)</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>BUY trim / SELL hedge</t>
-        </is>
+        <f>Расчеты!B25</f>
+        <v/>
+      </c>
+      <c r="D2">
+        <f>IF(C2="ESCAPE","СБРОС СТРУКТУРЫ",IF(C2="STRESS","СНИЗИТЬ РИСК И k","FLOW-РЕБАЛАНС"))</f>
+        <v/>
+      </c>
+      <c r="E2" s="5">
+        <f>ROUND(Расчеты!B24,2)</f>
+        <v/>
       </c>
       <c r="F2" s="5">
-        <f>IF(Расчеты!B17="НЕТ",0,MAX(0.01,ROUND(Расчеты!B19*Ввод!B19*Ввод!B23*0.5,2)))</f>
-        <v/>
-      </c>
-      <c r="G2">
-        <f>IF(AND(Расчеты!B11="ДА",F2&gt;0),"ЧАСТИЧНАЯ РЕБАЛАНСИРОВКА","ОЖИДАТЬ")</f>
+        <f>IF(C2="ESCAPE",0,ROUND(MAX(0.01,Ввод!B19*Ввод!B23),2))</f>
+        <v/>
+      </c>
+      <c r="G2" s="5">
+        <f>IF(A2="Цена вверх на Δ",ROUND(F2*0.40,2),ROUND(F2*0.60,2))</f>
         <v/>
       </c>
       <c r="H2" s="5">
-        <f>IF(F2=0,0,IF(OR(E2="BUY partial",E2="SELL partial"),ROUND(F2,2),ROUND(F2*0.6,2)))</f>
+        <f>IF(A2="Цена вверх на Δ",ROUND(F2*0.60,2),ROUND(F2*0.40,2))</f>
         <v/>
       </c>
       <c r="I2">
-        <f>IF(OR(Расчеты!B9="FAIL",Расчеты!B14&gt;Ввод!B22,Расчеты!B16&lt;-Ввод!B21),"ДА","НЕТ")</f>
+        <f>IF(AND(C2&lt;&gt;"ESCAPE",Расчеты!B11="ДА"),"ДА","НЕТ")</f>
         <v/>
       </c>
       <c r="J2">
-        <f>IF(I2="ДА","Риск превышен: survival/маржа/просадка","Нормальный цикл")</f>
-        <v/>
-      </c>
-      <c r="K2">
-        <f>IF(AND(F2&gt;0,I2="НЕТ"),"ДА","НЕТ")</f>
-        <v/>
-      </c>
-      <c r="L2">
-        <f>IF(K2="НЕТ","-",IF(D2="BUY (Рекомендации для выбранной BUY)","BUY","SELL"))</f>
-        <v/>
-      </c>
-      <c r="M2" s="5">
-        <f>IF(K2="НЕТ",0,ROUND(MAX(0.01,F2),2))</f>
-        <v/>
-      </c>
-      <c r="N2" s="7">
-        <f>IF(K2="НЕТ",0,B2)</f>
+        <f>IF(I2="НЕТ","-","SELL")</f>
+        <v/>
+      </c>
+      <c r="K2" s="5">
+        <f>IF(I2="НЕТ",0,ROUND(MAX(Ввод!B20,F2),2))</f>
+        <v/>
+      </c>
+      <c r="L2" s="7">
+        <f>IF(I2="НЕТ",0,B2)</f>
+        <v/>
+      </c>
+      <c r="M2">
+        <f>IF(C2="ESCAPE","Превышены лимиты риска",IF(C2="STRESS","Снизить k, ускорить сокращение риска","Плановый цикл"))</f>
+        <v/>
+      </c>
+      <c r="N2">
+        <f>IF(OR(Расчеты!B9="FAIL",Расчеты!B14&gt;Ввод!B22,Расчеты!B16&lt;-Ввод!B21),"ESCAPE","OK")</f>
         <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Цена вверх на Δ</t>
+          <t>Цена вниз на Δ</t>
         </is>
       </c>
       <c r="B3">
-        <f>Ввод!B12+Ввод!B18</f>
+        <f>Ввод!B12-Ввод!B18</f>
         <v/>
       </c>
       <c r="C3">
-        <f>IF(D3="BUY (Рекомендации для выбранной BUY)",Расчеты!B17,Расчеты!B18)</f>
-        <v/>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>SELL (Рекомендации для выбранной SELL)</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>SELL partial</t>
-        </is>
+        <f>Расчеты!B25</f>
+        <v/>
+      </c>
+      <c r="D3">
+        <f>IF(C3="ESCAPE","СБРОС СТРУКТУРЫ",IF(C3="STRESS","СНИЗИТЬ РИСК И k","FLOW-РЕБАЛАНС"))</f>
+        <v/>
+      </c>
+      <c r="E3" s="5">
+        <f>ROUND(Расчеты!B24,2)</f>
+        <v/>
       </c>
       <c r="F3" s="5">
-        <f>IF(Расчеты!B18="НЕТ",0,MAX(0.01,ROUND(Расчеты!B20*Ввод!B19*Ввод!B23*2,2)))</f>
-        <v/>
-      </c>
-      <c r="G3">
-        <f>IF(AND(Расчеты!B11="ДА",F3&gt;0),"ЧАСТИЧНАЯ РЕБАЛАНСИРОВКА","ОЖИДАТЬ")</f>
+        <f>IF(C3="ESCAPE",0,ROUND(MAX(0.01,Ввод!B19*Ввод!B23),2))</f>
+        <v/>
+      </c>
+      <c r="G3" s="5">
+        <f>IF(A3="Цена вверх на Δ",ROUND(F3*0.40,2),ROUND(F3*0.60,2))</f>
         <v/>
       </c>
       <c r="H3" s="5">
-        <f>IF(F3=0,0,IF(OR(E3="BUY partial",E3="SELL partial"),ROUND(F3,2),ROUND(F3*0.6,2)))</f>
+        <f>IF(A3="Цена вверх на Δ",ROUND(F3*0.60,2),ROUND(F3*0.40,2))</f>
         <v/>
       </c>
       <c r="I3">
-        <f>IF(OR(Расчеты!B9="FAIL",Расчеты!B14&gt;Ввод!B22,Расчеты!B16&lt;-Ввод!B21),"ДА","НЕТ")</f>
+        <f>IF(AND(C3&lt;&gt;"ESCAPE",Расчеты!B11="ДА"),"ДА","НЕТ")</f>
         <v/>
       </c>
       <c r="J3">
-        <f>IF(I3="ДА","Риск превышен: survival/маржа/просадка","Нормальный цикл")</f>
-        <v/>
-      </c>
-      <c r="K3">
-        <f>IF(AND(F3&gt;0,I3="НЕТ"),"ДА","НЕТ")</f>
-        <v/>
-      </c>
-      <c r="L3">
-        <f>IF(K3="НЕТ","-",IF(D3="BUY (Рекомендации для выбранной BUY)","BUY","SELL"))</f>
-        <v/>
-      </c>
-      <c r="M3" s="5">
-        <f>IF(K3="НЕТ",0,ROUND(MAX(0.01,F3),2))</f>
-        <v/>
-      </c>
-      <c r="N3" s="7">
-        <f>IF(K3="НЕТ",0,B3)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Цена вниз на Δ</t>
-        </is>
-      </c>
-      <c r="B4">
-        <f>Ввод!B12-Ввод!B18</f>
-        <v/>
-      </c>
-      <c r="C4">
-        <f>IF(D4="BUY (Рекомендации для выбранной BUY)",Расчеты!B17,Расчеты!B18)</f>
-        <v/>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>BUY (Рекомендации для выбранной BUY)</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>BUY partial</t>
-        </is>
-      </c>
-      <c r="F4" s="5">
-        <f>IF(Расчеты!B17="НЕТ",0,MAX(0.01,ROUND(Расчеты!B19*Ввод!B19*Ввод!B23*2,2)))</f>
-        <v/>
-      </c>
-      <c r="G4">
-        <f>IF(AND(Расчеты!B11="ДА",F4&gt;0),"ЧАСТИЧНАЯ РЕБАЛАНСИРОВКА","ОЖИДАТЬ")</f>
-        <v/>
-      </c>
-      <c r="H4" s="5">
-        <f>IF(F4=0,0,IF(OR(E4="BUY partial",E4="SELL partial"),ROUND(F4,2),ROUND(F4*0.6,2)))</f>
-        <v/>
-      </c>
-      <c r="I4">
-        <f>IF(OR(Расчеты!B9="FAIL",Расчеты!B14&gt;Ввод!B22,Расчеты!B16&lt;-Ввод!B21),"ДА","НЕТ")</f>
-        <v/>
-      </c>
-      <c r="J4">
-        <f>IF(I4="ДА","Риск превышен: survival/маржа/просадка","Нормальный цикл")</f>
-        <v/>
-      </c>
-      <c r="K4">
-        <f>IF(AND(F4&gt;0,I4="НЕТ"),"ДА","НЕТ")</f>
-        <v/>
-      </c>
-      <c r="L4">
-        <f>IF(K4="НЕТ","-",IF(D4="BUY (Рекомендации для выбранной BUY)","BUY","SELL"))</f>
-        <v/>
-      </c>
-      <c r="M4" s="5">
-        <f>IF(K4="НЕТ",0,ROUND(MAX(0.01,F4),2))</f>
-        <v/>
-      </c>
-      <c r="N4" s="7">
-        <f>IF(K4="НЕТ",0,B4)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Цена вниз на Δ</t>
-        </is>
-      </c>
-      <c r="B5">
-        <f>Ввод!B12-Ввод!B18</f>
-        <v/>
-      </c>
-      <c r="C5">
-        <f>IF(D5="BUY (Рекомендации для выбранной BUY)",Расчеты!B17,Расчеты!B18)</f>
-        <v/>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>SELL (Рекомендации для выбранной SELL)</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>SELL trim / BUY hedge</t>
-        </is>
-      </c>
-      <c r="F5" s="5">
-        <f>IF(Расчеты!B18="НЕТ",0,MAX(0.01,ROUND(Расчеты!B20*Ввод!B19*Ввод!B23*0.5,2)))</f>
-        <v/>
-      </c>
-      <c r="G5">
-        <f>IF(AND(Расчеты!B11="ДА",F5&gt;0),"ЧАСТИЧНАЯ РЕБАЛАНСИРОВКА","ОЖИДАТЬ")</f>
-        <v/>
-      </c>
-      <c r="H5" s="5">
-        <f>IF(F5=0,0,IF(OR(E5="BUY partial",E5="SELL partial"),ROUND(F5,2),ROUND(F5*0.6,2)))</f>
-        <v/>
-      </c>
-      <c r="I5">
-        <f>IF(OR(Расчеты!B9="FAIL",Расчеты!B14&gt;Ввод!B22,Расчеты!B16&lt;-Ввод!B21),"ДА","НЕТ")</f>
-        <v/>
-      </c>
-      <c r="J5">
-        <f>IF(I5="ДА","Риск превышен: survival/маржа/просадка","Нормальный цикл")</f>
-        <v/>
-      </c>
-      <c r="K5">
-        <f>IF(AND(F5&gt;0,I5="НЕТ"),"ДА","НЕТ")</f>
-        <v/>
-      </c>
-      <c r="L5">
-        <f>IF(K5="НЕТ","-",IF(D5="BUY (Рекомендации для выбранной BUY)","BUY","SELL"))</f>
-        <v/>
-      </c>
-      <c r="M5" s="5">
-        <f>IF(K5="НЕТ",0,ROUND(MAX(0.01,F5),2))</f>
-        <v/>
-      </c>
-      <c r="N5" s="7">
-        <f>IF(K5="НЕТ",0,B5)</f>
+        <f>IF(I3="НЕТ","-","SELL")</f>
+        <v/>
+      </c>
+      <c r="K3" s="5">
+        <f>IF(I3="НЕТ",0,ROUND(MAX(Ввод!B20,F3),2))</f>
+        <v/>
+      </c>
+      <c r="L3" s="7">
+        <f>IF(I3="НЕТ",0,B3)</f>
+        <v/>
+      </c>
+      <c r="M3">
+        <f>IF(C3="ESCAPE","Превышены лимиты риска",IF(C3="STRESS","Снизить k, ускорить сокращение риска","Плановый цикл"))</f>
+        <v/>
+      </c>
+      <c r="N3">
+        <f>IF(OR(Расчеты!B9="FAIL",Расчеты!B14&gt;Ввод!B22,Расчеты!B16&lt;-Ввод!B21),"ESCAPE","OK")</f>
         <v/>
       </c>
     </row>
@@ -8698,9 +8572,10 @@
         <f>IF(B2="ДА","ОТКРЫТЬ","ЖДАТЬ")</f>
         <v/>
       </c>
-      <c r="D2">
-        <f>IF(A2="Пробой вверх (+Δ)","BUY","SELL")</f>
-        <v/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
       </c>
       <c r="E2" s="5">
         <f>IF(C2&lt;&gt;"ОТКРЫТЬ",0,ROUND(MAX(0.01,MIN(Ввод!B20*0.01*Ввод!B23,(Ввод!B10*Ввод!B22/100-Расчеты!B13)*Ввод!B7/(Ввод!B6*Ввод!B12))),2))</f>
@@ -8737,9 +8612,10 @@
         <f>IF(B3="ДА","ОТКРЫТЬ","ЖДАТЬ")</f>
         <v/>
       </c>
-      <c r="D3">
-        <f>IF(A3="Пробой вверх (+Δ)","BUY","SELL")</f>
-        <v/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
       </c>
       <c r="E3" s="5">
         <f>IF(C3&lt;&gt;"ОТКРЫТЬ",0,ROUND(MAX(0.01,MIN(Ввод!B20*0.01*Ввод!B23,(Ввод!B10*Ввод!B22/100-Расчеты!B13)*Ввод!B7/(Ввод!B6*Ввод!B12))),2))</f>

</xml_diff>

<commit_message>
Align FSM formulas with reference and record final positive test verdict
</commit_message>
<xml_diff>
--- a/adaptive_ev_calculator.xlsx
+++ b/adaptive_ev_calculator.xlsx
@@ -8380,7 +8380,7 @@
         <v/>
       </c>
       <c r="F2" s="5">
-        <f>IF(C2="ESCAPE",0,ROUND(MAX(0.01,Ввод!B19*Ввод!B23),2))</f>
+        <f>IF(C2="ESCAPE",0,ROUND(MAX(0.01,MIN(Ввод!B19*Ввод!B23*E2,((Ввод!B10*Ввод!B22/100-Расчеты!B13)*Ввод!B7)/(Ввод!B6*MAX(B2,0.00001)))),2))</f>
         <v/>
       </c>
       <c r="G2" s="5">
@@ -8396,11 +8396,11 @@
         <v/>
       </c>
       <c r="J2">
-        <f>IF(I2="НЕТ","-","SELL")</f>
+        <f>IF(I2="НЕТ","-",IF(A2="Цена вверх на Δ","SELL","BUY"))</f>
         <v/>
       </c>
       <c r="K2" s="5">
-        <f>IF(I2="НЕТ",0,ROUND(MAX(Ввод!B20,F2),2))</f>
+        <f>IF(I2="НЕТ",0,ROUND(MAX(Ввод!B20,MIN(F2*1.2,((Ввод!B10*Ввод!B22/100-Расчеты!B13)*Ввод!B7)/(Ввод!B6*MAX(B2,0.00001)))),2))</f>
         <v/>
       </c>
       <c r="L2" s="7">
@@ -8439,7 +8439,7 @@
         <v/>
       </c>
       <c r="F3" s="5">
-        <f>IF(C3="ESCAPE",0,ROUND(MAX(0.01,Ввод!B19*Ввод!B23),2))</f>
+        <f>IF(C3="ESCAPE",0,ROUND(MAX(0.01,MIN(Ввод!B19*Ввод!B23*E3,((Ввод!B10*Ввод!B22/100-Расчеты!B13)*Ввод!B7)/(Ввод!B6*MAX(B3,0.00001)))),2))</f>
         <v/>
       </c>
       <c r="G3" s="5">
@@ -8455,11 +8455,11 @@
         <v/>
       </c>
       <c r="J3">
-        <f>IF(I3="НЕТ","-","SELL")</f>
+        <f>IF(I3="НЕТ","-",IF(A3="Цена вверх на Δ","SELL","BUY"))</f>
         <v/>
       </c>
       <c r="K3" s="5">
-        <f>IF(I3="НЕТ",0,ROUND(MAX(Ввод!B20,F3),2))</f>
+        <f>IF(I3="НЕТ",0,ROUND(MAX(Ввод!B20,MIN(F3*1.2,((Ввод!B10*Ввод!B22/100-Расчеты!B13)*Ввод!B7)/(Ввод!B6*MAX(B3,0.00001)))),2))</f>
         <v/>
       </c>
       <c r="L3" s="7">

</xml_diff>

<commit_message>
Add integral EV formulation and Excel EV proxy metrics
</commit_message>
<xml_diff>
--- a/adaptive_ev_calculator.xlsx
+++ b/adaptive_ev_calculator.xlsx
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B28"/>
+  <dimension ref="A1:B32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -753,6 +753,46 @@
       </c>
       <c r="B28" t="n">
         <v>5</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Edge drift μ (в цену/шаг)</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>3e-05</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Комиссия на 1 лот/шаг, USD</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Проскальзывание на 1 лот/шаг, USD</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Горизонт T (шаги)</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -7949,7 +7989,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:B30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -8246,6 +8286,61 @@
       </c>
       <c r="B25">
         <f>IF(OR(B14&gt;Ввод!B22,B16&lt;-Ввод!B21),"ESCAPE",IF(OR(B23&gt;0.7*Ввод!B27,B14&gt;0.7*Ввод!B22),"STRESS","FLOW"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Интеграл экспозиции ∫Qdt (proxy)</t>
+        </is>
+      </c>
+      <c r="B26">
+        <f>B15*Ввод!B32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Cost rate/шаг, USD (proxy)</t>
+        </is>
+      </c>
+      <c r="B27">
+        <f>ABS(B15)*(Ввод!B15*Ввод!B6 + Ввод!B30 + Ввод!B31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Интеграл издержек ∫Cost dt</t>
+        </is>
+      </c>
+      <c r="B28">
+        <f>B27*Ввод!B32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>EV(T) = μ∫Qdt - ∫Costdt</t>
+        </is>
+      </c>
+      <c r="B29">
+        <f>Ввод!B29*B26 - B28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Условие +EV</t>
+        </is>
+      </c>
+      <c r="B30">
+        <f>IF(B29&gt;0,"YES","NO")</f>
         <v/>
       </c>
     </row>

</xml_diff>